<commit_message>
added tests in junit
</commit_message>
<xml_diff>
--- a/docs/Lab02/vtir3660_Lab02_BBT_TCs_Form.xlsx
+++ b/docs/Lab02/vtir3660_Lab02_BBT_TCs_Form.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\info\csubb\Semestru 6\VVSS\lab\lab1\MyDrinkShop\docs\Lab02\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\vvss-lab\docs\Lab02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CD9E6EE-19DF-416D-8216-766C73755384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054EA6D8-0E6D-4D49-943A-AE24BC0D2174}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19200" yWindow="0" windowWidth="19200" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statement" sheetId="1" r:id="rId1"/>
@@ -318,9 +318,6 @@
     <t>Executable</t>
   </si>
   <si>
-    <t>id is int, id in [1, 9999]</t>
-  </si>
-  <si>
     <t>01. id = 0, below min</t>
   </si>
   <si>
@@ -490,6 +487,9 @@
   </si>
   <si>
     <t>11. nume = "A…256chars", length = 256</t>
+  </si>
+  <si>
+    <t>Date valide (Preț în intervalul [0.01, 10000], Nume cu lungime [3, 50])</t>
   </si>
 </sst>
 </file>
@@ -1167,14 +1167,61 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1182,14 +1229,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1197,7 +1236,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1206,7 +1244,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1214,94 +1251,57 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1611,36 +1611,36 @@
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A1:O26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="22.5546875" customWidth="1"/>
-    <col min="9" max="9" width="32.88671875" customWidth="1"/>
-    <col min="10" max="10" width="10.5546875" customWidth="1"/>
-    <col min="12" max="12" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" customWidth="1"/>
+    <col min="9" max="9" width="32.85546875" customWidth="1"/>
+    <col min="10" max="10" width="10.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.140625" customWidth="1"/>
     <col min="14" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="C1" s="56" t="s">
+    <row r="1" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="C1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="57"/>
-      <c r="E1" s="57"/>
-      <c r="F1" s="55"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="53"/>
       <c r="H1" s="51" t="s">
         <v>45</v>
       </c>
       <c r="I1" s="51"/>
       <c r="J1" s="51"/>
     </row>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H2" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="J2" s="55"/>
-    </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="I2" s="80"/>
+      <c r="J2" s="53"/>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
         <v>47</v>
@@ -1649,7 +1649,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H4" s="2" t="s">
         <v>49</v>
       </c>
@@ -1658,14 +1658,14 @@
       </c>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="H5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="37"/>
       <c r="H6" s="2" t="s">
         <v>52</v>
@@ -1673,50 +1673,50 @@
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
     </row>
-    <row r="7" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="49" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>1</v>
       </c>
@@ -1724,32 +1724,32 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B18" s="49" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C20" s="47" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>60</v>
       </c>
@@ -1766,7 +1766,7 @@
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>61</v>
       </c>
@@ -1783,25 +1783,25 @@
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
     </row>
-    <row r="24" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="48"/>
       <c r="B24" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="C24" s="86"/>
-      <c r="D24" s="86"/>
-      <c r="E24" s="86"/>
-      <c r="F24" s="86"/>
-      <c r="G24" s="86"/>
-      <c r="H24" s="86"/>
-      <c r="I24" s="86"/>
-      <c r="J24" s="86"/>
-      <c r="K24" s="86"/>
-      <c r="L24" s="86"/>
-      <c r="M24" s="86"/>
-      <c r="N24" s="86"/>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
+      <c r="G24" s="64"/>
+      <c r="H24" s="64"/>
+      <c r="I24" s="64"/>
+      <c r="J24" s="64"/>
+      <c r="K24" s="64"/>
+      <c r="L24" s="64"/>
+      <c r="M24" s="64"/>
+      <c r="N24" s="64"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C26" s="50"/>
     </row>
   </sheetData>
@@ -1821,63 +1821,63 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:Q22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.88671875" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.85546875" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="29.44140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29.42578125" customWidth="1"/>
     <col min="17" max="17" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B1" s="56" t="s">
+    <row r="1" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="55"/>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B3" s="94" t="s">
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="53"/>
+    </row>
+    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B3" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="55"/>
-    </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="53"/>
+    </row>
+    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="55"/>
-      <c r="G5" s="99" t="s">
+      <c r="C5" s="80"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="53"/>
+      <c r="G5" s="97" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
-      <c r="P5" s="57"/>
-      <c r="Q5" s="55"/>
-    </row>
-    <row r="6" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="80"/>
+      <c r="N5" s="80"/>
+      <c r="O5" s="80"/>
+      <c r="P5" s="80"/>
+      <c r="Q5" s="53"/>
+    </row>
+    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6" s="23" t="s">
         <v>4</v>
       </c>
@@ -1890,27 +1890,27 @@
       <c r="E6" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="67" t="s">
+      <c r="H6" s="85" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="67" t="s">
+      <c r="I6" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="57"/>
-      <c r="K6" s="57"/>
-      <c r="L6" s="57"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="55"/>
-      <c r="P6" s="67" t="s">
+      <c r="J6" s="80"/>
+      <c r="K6" s="80"/>
+      <c r="L6" s="80"/>
+      <c r="M6" s="80"/>
+      <c r="N6" s="80"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="Q6" s="55"/>
-    </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="Q6" s="53"/>
+    </row>
+    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="4">
         <v>1</v>
       </c>
@@ -1921,8 +1921,8 @@
         <v>12</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
       <c r="I7" s="23" t="s">
         <v>13</v>
       </c>
@@ -1938,18 +1938,18 @@
       <c r="M7" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="67"/>
-      <c r="O7" s="55"/>
-      <c r="P7" s="67" t="s">
+      <c r="N7" s="85"/>
+      <c r="O7" s="53"/>
+      <c r="P7" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="Q7" s="55"/>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="Q7" s="53"/>
+    </row>
+    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="61"/>
+      <c r="C8" s="66"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4" t="s">
         <v>19</v>
@@ -1976,13 +1976,13 @@
         <v>23</v>
       </c>
       <c r="N8" s="93"/>
-      <c r="O8" s="55"/>
+      <c r="O8" s="53"/>
       <c r="P8" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="Q8" s="55"/>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="Q8" s="53"/>
+    </row>
+    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B9" s="4">
         <v>3</v>
       </c>
@@ -2015,17 +2015,17 @@
         <v>28</v>
       </c>
       <c r="N9" s="93"/>
-      <c r="O9" s="55"/>
+      <c r="O9" s="53"/>
       <c r="P9" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="Q9" s="55"/>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="Q9" s="53"/>
+    </row>
+    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="61"/>
+      <c r="C10" s="66"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>29</v>
@@ -2049,14 +2049,14 @@
       <c r="M10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="N10" s="100"/>
-      <c r="O10" s="55"/>
-      <c r="P10" s="100" t="s">
+      <c r="N10" s="94"/>
+      <c r="O10" s="53"/>
+      <c r="P10" s="94" t="s">
         <v>31</v>
       </c>
-      <c r="Q10" s="55"/>
-    </row>
-    <row r="11" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q10" s="53"/>
+    </row>
+    <row r="11" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4">
         <v>5</v>
       </c>
@@ -2088,18 +2088,18 @@
       <c r="M11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="N11" s="100"/>
-      <c r="O11" s="55"/>
-      <c r="P11" s="100" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q11" s="55"/>
-    </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="N11" s="94"/>
+      <c r="O11" s="53"/>
+      <c r="P11" s="94" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q11" s="53"/>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="61"/>
+      <c r="C12" s="66"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>35</v>
@@ -2127,12 +2127,12 @@
       </c>
       <c r="N12" s="9"/>
       <c r="O12" s="9"/>
-      <c r="P12" s="97" t="s">
+      <c r="P12" s="98" t="s">
         <v>38</v>
       </c>
-      <c r="Q12" s="55"/>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="Q12" s="53"/>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" s="4">
         <v>7</v>
       </c>
@@ -2164,18 +2164,18 @@
       <c r="M13" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="N13" s="97"/>
-      <c r="O13" s="55"/>
-      <c r="P13" s="97" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="55"/>
-    </row>
-    <row r="14" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="N13" s="98"/>
+      <c r="O13" s="53"/>
+      <c r="P13" s="98" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q13" s="53"/>
+    </row>
+    <row r="14" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B14" s="4">
         <v>8</v>
       </c>
-      <c r="C14" s="61"/>
+      <c r="C14" s="66"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
         <v>40</v>
@@ -2201,12 +2201,12 @@
       <c r="M14" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="N14" s="101"/>
-      <c r="O14" s="55"/>
-      <c r="P14" s="96"/>
-      <c r="Q14" s="55"/>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="N14" s="100"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="99"/>
+      <c r="Q14" s="53"/>
+    </row>
+    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="4">
         <v>9</v>
       </c>
@@ -2229,17 +2229,17 @@
       <c r="L15" s="18"/>
       <c r="M15" s="18"/>
       <c r="N15" s="93"/>
-      <c r="O15" s="55"/>
-      <c r="P15" s="96" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q15" s="55"/>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O15" s="53"/>
+      <c r="P15" s="99" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" s="53"/>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" s="4">
         <v>10</v>
       </c>
-      <c r="C16" s="61"/>
+      <c r="C16" s="66"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
         <v>43</v>
@@ -2252,11 +2252,11 @@
       <c r="L16" s="18"/>
       <c r="M16" s="18"/>
       <c r="N16" s="93"/>
-      <c r="O16" s="55"/>
-      <c r="P16" s="96"/>
-      <c r="Q16" s="55"/>
-    </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O16" s="53"/>
+      <c r="P16" s="99"/>
+      <c r="Q16" s="53"/>
+    </row>
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="4">
         <v>11</v>
       </c>
@@ -2273,15 +2273,15 @@
       <c r="L17" s="18"/>
       <c r="M17" s="18"/>
       <c r="N17" s="93"/>
-      <c r="O17" s="55"/>
-      <c r="P17" s="96"/>
-      <c r="Q17" s="55"/>
-    </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O17" s="53"/>
+      <c r="P17" s="99"/>
+      <c r="Q17" s="53"/>
+    </row>
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="4">
         <v>12</v>
       </c>
-      <c r="C18" s="61"/>
+      <c r="C18" s="66"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="G18" s="19"/>
@@ -2292,11 +2292,11 @@
       <c r="L18" s="18"/>
       <c r="M18" s="18"/>
       <c r="N18" s="93"/>
-      <c r="O18" s="55"/>
-      <c r="P18" s="96"/>
-      <c r="Q18" s="55"/>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O18" s="53"/>
+      <c r="P18" s="99"/>
+      <c r="Q18" s="53"/>
+    </row>
+    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B19" s="4">
         <v>13</v>
       </c>
@@ -2313,36 +2313,43 @@
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="93"/>
-      <c r="O19" s="55"/>
-      <c r="P19" s="96"/>
-      <c r="Q19" s="55"/>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.3">
+      <c r="O19" s="53"/>
+      <c r="P19" s="99"/>
+      <c r="Q19" s="53"/>
+    </row>
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="4">
         <v>14</v>
       </c>
-      <c r="C20" s="61"/>
+      <c r="C20" s="66"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
         <v>44</v>
       </c>
-      <c r="F22" s="98"/>
-      <c r="G22" s="86"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N7:O7"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="N15:O15"/>
+    <mergeCell ref="P15:Q15"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="P9:Q9"/>
     <mergeCell ref="F22:G22"/>
     <mergeCell ref="G5:Q5"/>
     <mergeCell ref="N19:O19"/>
@@ -2359,22 +2366,15 @@
     <mergeCell ref="P7:Q7"/>
     <mergeCell ref="P16:Q16"/>
     <mergeCell ref="N10:O10"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="N15:O15"/>
-    <mergeCell ref="P15:Q15"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N7:O7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2386,68 +2386,68 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:R30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
-    <col min="6" max="6" width="5.5546875" customWidth="1"/>
-    <col min="7" max="7" width="9.44140625" customWidth="1"/>
+    <col min="6" max="6" width="5.5703125" customWidth="1"/>
+    <col min="7" max="7" width="9.42578125" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5546875" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="23.33203125" customWidth="1"/>
-    <col min="18" max="18" width="9.44140625" customWidth="1"/>
+    <col min="10" max="10" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5703125" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="23.28515625" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B1" s="56" t="s">
+    <row r="1" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="55"/>
-    </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B3" s="94" t="s">
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="53"/>
+    </row>
+    <row r="3" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B3" s="101" t="s">
         <v>63</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="55"/>
-    </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B5" s="108" t="s">
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="53"/>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B5" s="106" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="55"/>
+      <c r="C5" s="80"/>
+      <c r="D5" s="53"/>
       <c r="E5" s="3"/>
-      <c r="G5" s="99" t="s">
+      <c r="G5" s="97" t="s">
         <v>65</v>
       </c>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
-      <c r="L5" s="57"/>
-      <c r="M5" s="57"/>
-      <c r="N5" s="57"/>
-      <c r="O5" s="57"/>
-      <c r="P5" s="57"/>
-      <c r="Q5" s="57"/>
-      <c r="R5" s="55"/>
-    </row>
-    <row r="6" spans="2:18" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="80"/>
+      <c r="N5" s="80"/>
+      <c r="O5" s="80"/>
+      <c r="P5" s="80"/>
+      <c r="Q5" s="80"/>
+      <c r="R5" s="53"/>
+    </row>
+    <row r="6" spans="2:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>66</v>
       </c>
@@ -2458,45 +2458,45 @@
         <v>64</v>
       </c>
       <c r="E6" s="10"/>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="65" t="s">
         <v>67</v>
       </c>
-      <c r="H6" s="60" t="s">
+      <c r="H6" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="65" t="s">
         <v>69</v>
       </c>
-      <c r="J6" s="67" t="s">
+      <c r="J6" s="85" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="109" t="s">
+      <c r="K6" s="107" t="s">
         <v>10</v>
       </c>
-      <c r="L6" s="57"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="55"/>
-      <c r="Q6" s="109" t="s">
+      <c r="L6" s="80"/>
+      <c r="M6" s="80"/>
+      <c r="N6" s="80"/>
+      <c r="O6" s="80"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="R6" s="55"/>
-    </row>
-    <row r="7" spans="2:18" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R6" s="53"/>
+    </row>
+    <row r="7" spans="2:18" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="95">
         <v>1</v>
       </c>
       <c r="C7" s="105" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G7" s="61"/>
-      <c r="H7" s="61"/>
-      <c r="I7" s="61"/>
-      <c r="J7" s="61"/>
+      <c r="G7" s="66"/>
+      <c r="H7" s="66"/>
+      <c r="I7" s="66"/>
+      <c r="J7" s="66"/>
       <c r="K7" s="23" t="s">
         <v>13</v>
       </c>
@@ -2513,16 +2513,16 @@
         <v>17</v>
       </c>
       <c r="P7" s="23"/>
-      <c r="Q7" s="67" t="s">
+      <c r="Q7" s="85" t="s">
+        <v>72</v>
+      </c>
+      <c r="R7" s="53"/>
+    </row>
+    <row r="8" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B8" s="104"/>
+      <c r="C8" s="104"/>
+      <c r="D8" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="R7" s="55"/>
-    </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B8" s="106"/>
-      <c r="C8" s="106"/>
-      <c r="D8" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="G8" s="23">
         <v>1</v>
@@ -2531,7 +2531,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J8" s="16"/>
       <c r="K8" s="34"/>
@@ -2541,13 +2541,13 @@
       <c r="O8" s="34"/>
       <c r="P8" s="34"/>
       <c r="Q8" s="103"/>
-      <c r="R8" s="55"/>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B9" s="106"/>
-      <c r="C9" s="106"/>
+      <c r="R8" s="53"/>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B9" s="104"/>
+      <c r="C9" s="104"/>
       <c r="D9" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G9" s="19">
         <v>2</v>
@@ -2557,7 +2557,7 @@
       </c>
       <c r="I9" s="21"/>
       <c r="J9" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K9" s="22" t="s">
         <v>41</v>
@@ -2573,16 +2573,16 @@
         <v>27</v>
       </c>
       <c r="P9" s="18"/>
-      <c r="Q9" s="97" t="s">
+      <c r="Q9" s="98" t="s">
+        <v>77</v>
+      </c>
+      <c r="R9" s="53"/>
+    </row>
+    <row r="10" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B10" s="104"/>
+      <c r="C10" s="104"/>
+      <c r="D10" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="R9" s="55"/>
-    </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B10" s="106"/>
-      <c r="C10" s="106"/>
-      <c r="D10" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="G10" s="23">
         <v>3</v>
@@ -2596,28 +2596,28 @@
         <v>1</v>
       </c>
       <c r="L10" s="34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="M10" s="34">
         <v>0.01</v>
       </c>
       <c r="N10" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="O10" s="34" t="s">
         <v>81</v>
-      </c>
-      <c r="O10" s="34" t="s">
-        <v>82</v>
       </c>
       <c r="P10" s="34"/>
       <c r="Q10" s="103" t="s">
         <v>24</v>
       </c>
-      <c r="R10" s="55"/>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B11" s="106"/>
-      <c r="C11" s="106"/>
+      <c r="R10" s="53"/>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B11" s="104"/>
+      <c r="C11" s="104"/>
       <c r="D11" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G11" s="23">
         <v>4</v>
@@ -2631,7 +2631,7 @@
         <v>9999</v>
       </c>
       <c r="L11" s="34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M11" s="34">
         <v>999999.99</v>
@@ -2646,13 +2646,13 @@
       <c r="Q11" s="103" t="s">
         <v>24</v>
       </c>
-      <c r="R11" s="55"/>
-    </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
+      <c r="R11" s="53"/>
+    </row>
+    <row r="12" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B12" s="66"/>
+      <c r="C12" s="66"/>
       <c r="D12" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G12" s="23">
         <v>5</v>
@@ -2666,7 +2666,7 @@
         <v>9998</v>
       </c>
       <c r="L12" s="34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="M12" s="34">
         <v>999999.98</v>
@@ -2681,9 +2681,9 @@
       <c r="Q12" s="103" t="s">
         <v>24</v>
       </c>
-      <c r="R12" s="55"/>
-    </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="R12" s="53"/>
+    </row>
+    <row r="13" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B13" s="95">
         <v>2</v>
       </c>
@@ -2691,7 +2691,7 @@
         <v>25</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G13" s="19">
         <v>6</v>
@@ -2701,13 +2701,13 @@
       </c>
       <c r="I13" s="21"/>
       <c r="J13" s="21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K13" s="22">
         <v>10000</v>
       </c>
       <c r="L13" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M13" s="18">
         <v>1000000</v>
@@ -2719,16 +2719,16 @@
         <v>23</v>
       </c>
       <c r="P13" s="18"/>
-      <c r="Q13" s="97" t="s">
+      <c r="Q13" s="98" t="s">
+        <v>88</v>
+      </c>
+      <c r="R13" s="53"/>
+    </row>
+    <row r="14" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B14" s="104"/>
+      <c r="C14" s="104"/>
+      <c r="D14" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="R13" s="55"/>
-    </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B14" s="106"/>
-      <c r="C14" s="106"/>
-      <c r="D14" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="G14" s="23">
         <v>7</v>
@@ -2749,13 +2749,13 @@
       <c r="O14" s="34"/>
       <c r="P14" s="34"/>
       <c r="Q14" s="103"/>
-      <c r="R14" s="55"/>
-    </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B15" s="106"/>
-      <c r="C15" s="106"/>
+      <c r="R14" s="53"/>
+    </row>
+    <row r="15" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B15" s="104"/>
+      <c r="C15" s="104"/>
       <c r="D15" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G15" s="23">
         <v>8</v>
@@ -2776,13 +2776,13 @@
       <c r="O15" s="34"/>
       <c r="P15" s="34"/>
       <c r="Q15" s="103"/>
-      <c r="R15" s="55"/>
-    </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B16" s="106"/>
-      <c r="C16" s="106"/>
+      <c r="R15" s="53"/>
+    </row>
+    <row r="16" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B16" s="104"/>
+      <c r="C16" s="104"/>
       <c r="D16" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G16" s="23">
         <v>9</v>
@@ -2797,13 +2797,13 @@
       <c r="O16" s="34"/>
       <c r="P16" s="34"/>
       <c r="Q16" s="103"/>
-      <c r="R16" s="55"/>
-    </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B17" s="106"/>
-      <c r="C17" s="106"/>
+      <c r="R16" s="53"/>
+    </row>
+    <row r="17" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B17" s="104"/>
+      <c r="C17" s="104"/>
       <c r="D17" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G17" s="23">
         <v>10</v>
@@ -2818,13 +2818,13 @@
       <c r="O17" s="34"/>
       <c r="P17" s="34"/>
       <c r="Q17" s="103"/>
-      <c r="R17" s="55"/>
-    </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B18" s="61"/>
-      <c r="C18" s="61"/>
+      <c r="R17" s="53"/>
+    </row>
+    <row r="18" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B18" s="66"/>
+      <c r="C18" s="66"/>
       <c r="D18" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G18" s="23">
         <v>11</v>
@@ -2839,17 +2839,17 @@
       <c r="O18" s="34"/>
       <c r="P18" s="34"/>
       <c r="Q18" s="103"/>
-      <c r="R18" s="55"/>
-    </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="R18" s="53"/>
+    </row>
+    <row r="19" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B19" s="95">
         <v>3</v>
       </c>
       <c r="C19" s="105" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="G19" s="23">
         <v>12</v>
@@ -2864,13 +2864,13 @@
       <c r="O19" s="34"/>
       <c r="P19" s="34"/>
       <c r="Q19" s="103"/>
-      <c r="R19" s="55"/>
-    </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B20" s="106"/>
-      <c r="C20" s="106"/>
+      <c r="R19" s="53"/>
+    </row>
+    <row r="20" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B20" s="104"/>
+      <c r="C20" s="104"/>
       <c r="D20" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G20" s="23">
         <v>13</v>
@@ -2885,13 +2885,13 @@
       <c r="O20" s="34"/>
       <c r="P20" s="34"/>
       <c r="Q20" s="103"/>
-      <c r="R20" s="55"/>
-    </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B21" s="106"/>
-      <c r="C21" s="106"/>
+      <c r="R20" s="53"/>
+    </row>
+    <row r="21" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B21" s="104"/>
+      <c r="C21" s="104"/>
       <c r="D21" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G21" s="23">
         <v>14</v>
@@ -2906,13 +2906,13 @@
       <c r="O21" s="34"/>
       <c r="P21" s="34"/>
       <c r="Q21" s="103"/>
-      <c r="R21" s="55"/>
-    </row>
-    <row r="22" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B22" s="106"/>
-      <c r="C22" s="106"/>
+      <c r="R21" s="53"/>
+    </row>
+    <row r="22" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B22" s="104"/>
+      <c r="C22" s="104"/>
       <c r="D22" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G22" s="23">
         <v>15</v>
@@ -2927,13 +2927,13 @@
       <c r="O22" s="34"/>
       <c r="P22" s="34"/>
       <c r="Q22" s="103"/>
-      <c r="R22" s="55"/>
-    </row>
-    <row r="23" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B23" s="106"/>
-      <c r="C23" s="106"/>
+      <c r="R22" s="53"/>
+    </row>
+    <row r="23" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B23" s="104"/>
+      <c r="C23" s="104"/>
       <c r="D23" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G23" s="23">
         <v>16</v>
@@ -2948,13 +2948,13 @@
       <c r="O23" s="34"/>
       <c r="P23" s="34"/>
       <c r="Q23" s="103"/>
-      <c r="R23" s="55"/>
-    </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B24" s="61"/>
-      <c r="C24" s="61"/>
+      <c r="R23" s="53"/>
+    </row>
+    <row r="24" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B24" s="66"/>
+      <c r="C24" s="66"/>
       <c r="D24" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G24" s="23">
         <v>17</v>
@@ -2969,9 +2969,9 @@
       <c r="O24" s="34"/>
       <c r="P24" s="34"/>
       <c r="Q24" s="103"/>
-      <c r="R24" s="55"/>
-    </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.3">
+      <c r="R24" s="53"/>
+    </row>
+    <row r="25" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B25" s="95">
         <v>4</v>
       </c>
@@ -2994,83 +2994,59 @@
       <c r="O25" s="34"/>
       <c r="P25" s="34"/>
       <c r="Q25" s="103"/>
-      <c r="R25" s="55"/>
-    </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B26" s="106"/>
-      <c r="C26" s="106"/>
+      <c r="R25" s="53"/>
+    </row>
+    <row r="26" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B26" s="104"/>
+      <c r="C26" s="104"/>
       <c r="D26" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B27" s="106"/>
-      <c r="C27" s="106"/>
+    <row r="27" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B27" s="104"/>
+      <c r="C27" s="104"/>
       <c r="D27" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B28" s="106"/>
-      <c r="C28" s="106"/>
+    <row r="28" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B28" s="104"/>
+      <c r="C28" s="104"/>
       <c r="D28" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="98"/>
-      <c r="H28" s="86"/>
-      <c r="I28" s="107"/>
-      <c r="J28" s="86"/>
-      <c r="K28" s="86"/>
-      <c r="L28" s="86"/>
-      <c r="M28" s="86"/>
+      <c r="G28" s="96"/>
+      <c r="H28" s="64"/>
+      <c r="I28" s="109"/>
+      <c r="J28" s="64"/>
+      <c r="K28" s="64"/>
+      <c r="L28" s="64"/>
+      <c r="M28" s="64"/>
       <c r="N28" s="43"/>
     </row>
-    <row r="29" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B29" s="106"/>
-      <c r="C29" s="106"/>
+    <row r="29" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B29" s="104"/>
+      <c r="C29" s="104"/>
       <c r="D29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="I29" s="104"/>
-      <c r="J29" s="86"/>
-      <c r="K29" s="86"/>
-      <c r="L29" s="86"/>
-      <c r="M29" s="86"/>
+      <c r="I29" s="108"/>
+      <c r="J29" s="64"/>
+      <c r="K29" s="64"/>
+      <c r="L29" s="64"/>
+      <c r="M29" s="64"/>
       <c r="N29" s="44"/>
     </row>
-    <row r="30" spans="2:18" x14ac:dyDescent="0.3">
-      <c r="B30" s="61"/>
-      <c r="C30" s="61"/>
+    <row r="30" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B30" s="66"/>
+      <c r="C30" s="66"/>
       <c r="D30" s="2" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="Q9:R9"/>
-    <mergeCell ref="B7:B12"/>
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="Q8:R8"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="B19:B24"/>
-    <mergeCell ref="C19:C24"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="Q7:R7"/>
-    <mergeCell ref="Q25:R25"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B13:B18"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q6:R6"/>
-    <mergeCell ref="K6:P6"/>
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="Q17:R17"/>
@@ -3087,6 +3063,30 @@
     <mergeCell ref="Q10:R10"/>
     <mergeCell ref="G28:H28"/>
     <mergeCell ref="I28:M28"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B13:B18"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="K6:P6"/>
+    <mergeCell ref="B25:B30"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="Q24:R24"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="Q23:R23"/>
+    <mergeCell ref="B19:B24"/>
+    <mergeCell ref="C19:C24"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="Q25:R25"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="Q21:R21"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="Q22:R22"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="B7:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -3100,75 +3100,75 @@
     <tabColor theme="7" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="B1:P21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.88671875" customWidth="1"/>
-    <col min="13" max="13" width="30.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.85546875" customWidth="1"/>
+    <col min="13" max="13" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B1" s="56" t="s">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B1" s="79" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="57"/>
-      <c r="D1" s="57"/>
-      <c r="E1" s="55"/>
-    </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B3" s="72" t="s">
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="53"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B3" s="89" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="80"/>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="53"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B4" s="81" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="57"/>
-      <c r="H3" s="57"/>
-      <c r="I3" s="57"/>
-      <c r="J3" s="57"/>
-      <c r="K3" s="57"/>
-      <c r="L3" s="57"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="55"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B4" s="58" t="s">
+      <c r="C4" s="54" t="s">
         <v>102</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="D4" s="74" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="90" t="s">
+      <c r="E4" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="84" t="s">
-        <v>105</v>
-      </c>
-      <c r="F4" s="67" t="s">
+      <c r="F4" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="57"/>
-      <c r="H4" s="57"/>
-      <c r="I4" s="57"/>
-      <c r="J4" s="57"/>
-      <c r="K4" s="57"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="67" t="s">
+      <c r="G4" s="80"/>
+      <c r="H4" s="80"/>
+      <c r="I4" s="80"/>
+      <c r="J4" s="80"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="53"/>
+      <c r="M4" s="85" t="s">
         <v>11</v>
       </c>
-      <c r="N4" s="55"/>
-    </row>
-    <row r="5" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="59"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="91"/>
-      <c r="E5" s="59"/>
+      <c r="N4" s="53"/>
+    </row>
+    <row r="5" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="62"/>
+      <c r="C5" s="55"/>
+      <c r="D5" s="75"/>
+      <c r="E5" s="62"/>
       <c r="F5" s="26" t="s">
         <v>13</v>
       </c>
@@ -3184,27 +3184,27 @@
       <c r="J5" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="84"/>
-      <c r="L5" s="71"/>
+      <c r="K5" s="61"/>
+      <c r="L5" s="68"/>
       <c r="M5" s="26" t="s">
         <v>18</v>
       </c>
       <c r="N5" s="26" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="6" spans="2:14" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B6" s="24">
         <v>1</v>
       </c>
-      <c r="C6" s="88" t="s">
+      <c r="C6" s="69" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="E6" s="24" t="s">
         <v>108</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>109</v>
       </c>
       <c r="F6" s="29">
         <v>101</v>
@@ -3221,8 +3221,8 @@
       <c r="J6" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="K6" s="63"/>
-      <c r="L6" s="64"/>
+      <c r="K6" s="82"/>
+      <c r="L6" s="83"/>
       <c r="M6" s="29" t="s">
         <v>24</v>
       </c>
@@ -3230,17 +3230,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="12">
         <f t="shared" ref="B7:B13" si="0">B6+1</f>
         <v>2</v>
       </c>
-      <c r="C7" s="89"/>
+      <c r="C7" s="70"/>
       <c r="D7" s="31" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F7" s="8">
         <v>102</v>
@@ -3255,8 +3255,8 @@
       <c r="J7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="54"/>
-      <c r="L7" s="55"/>
+      <c r="K7" s="78"/>
+      <c r="L7" s="53"/>
       <c r="M7" s="8" t="s">
         <v>31</v>
       </c>
@@ -3264,17 +3264,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="12">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C8" s="89"/>
+      <c r="C8" s="70"/>
       <c r="D8" s="31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F8" s="6">
         <v>103</v>
@@ -3300,12 +3300,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="12">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C9" s="89"/>
+      <c r="C9" s="70"/>
       <c r="D9" s="31" t="s">
         <v>27</v>
       </c>
@@ -3327,8 +3327,8 @@
       <c r="J9" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="87"/>
-      <c r="L9" s="55"/>
+      <c r="K9" s="67"/>
+      <c r="L9" s="53"/>
       <c r="M9" s="12" t="s">
         <v>27</v>
       </c>
@@ -3336,35 +3336,35 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="12">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C10" s="89"/>
+      <c r="C10" s="70"/>
       <c r="D10" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F10" s="15">
         <v>1</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H10" s="11">
         <v>0.01</v>
       </c>
       <c r="I10" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="J10" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="K10" s="62"/>
-      <c r="L10" s="55"/>
+      <c r="K10" s="73"/>
+      <c r="L10" s="53"/>
       <c r="M10" s="6" t="s">
         <v>24</v>
       </c>
@@ -3372,23 +3372,23 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B11" s="12">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C11" s="89"/>
+      <c r="C11" s="70"/>
       <c r="D11" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F11" s="15">
         <v>9999</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H11" s="11">
         <v>999999.99</v>
@@ -3399,8 +3399,8 @@
       <c r="J11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K11" s="62"/>
-      <c r="L11" s="55"/>
+      <c r="K11" s="73"/>
+      <c r="L11" s="53"/>
       <c r="M11" s="5" t="s">
         <v>24</v>
       </c>
@@ -3408,23 +3408,23 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="12">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C12" s="89"/>
+      <c r="C12" s="70"/>
       <c r="D12" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F12" s="15">
         <v>9998</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H12" s="11">
         <v>999999.98</v>
@@ -3435,8 +3435,8 @@
       <c r="J12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="K12" s="62"/>
-      <c r="L12" s="55"/>
+      <c r="K12" s="73"/>
+      <c r="L12" s="53"/>
       <c r="M12" s="5" t="s">
         <v>24</v>
       </c>
@@ -3444,12 +3444,12 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="25">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C13" s="81"/>
+      <c r="C13" s="55"/>
       <c r="D13" s="32" t="s">
         <v>27</v>
       </c>
@@ -3471,8 +3471,8 @@
       <c r="J13" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="K13" s="70"/>
-      <c r="L13" s="71"/>
+      <c r="K13" s="88"/>
+      <c r="L13" s="68"/>
       <c r="M13" s="25" t="s">
         <v>27</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="2:14" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:14" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B14" s="27"/>
       <c r="C14" s="27"/>
       <c r="D14" s="28"/>
@@ -3495,9 +3495,9 @@
       <c r="M14" s="27"/>
       <c r="N14" s="27"/>
     </row>
-    <row r="15" spans="2:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:14" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="27" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C15" s="27"/>
       <c r="D15" s="28"/>
@@ -3507,102 +3507,102 @@
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
       <c r="J15" s="7"/>
-      <c r="K15" s="85"/>
-      <c r="L15" s="86"/>
+      <c r="K15" s="63"/>
+      <c r="L15" s="64"/>
       <c r="M15" s="7"/>
     </row>
-    <row r="16" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="M16" s="7"/>
     </row>
-    <row r="17" spans="2:16" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="75" t="s">
+    <row r="17" spans="2:16" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="58" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="39" t="s">
         <v>116</v>
       </c>
-      <c r="D17" s="76"/>
-      <c r="E17" s="76"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="39" t="s">
+      <c r="H17" s="58" t="s">
         <v>117</v>
       </c>
-      <c r="H17" s="75" t="s">
+      <c r="I17" s="59"/>
+      <c r="J17" s="59"/>
+      <c r="K17" s="59"/>
+      <c r="L17" s="60"/>
+      <c r="M17" s="58" t="s">
         <v>118</v>
       </c>
-      <c r="I17" s="76"/>
-      <c r="J17" s="76"/>
-      <c r="K17" s="76"/>
-      <c r="L17" s="77"/>
-      <c r="M17" s="75" t="s">
+      <c r="N17" s="59"/>
+      <c r="O17" s="59"/>
+      <c r="P17" s="60"/>
+    </row>
+    <row r="18" spans="2:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="56" t="s">
+        <v>102</v>
+      </c>
+      <c r="C18" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="N17" s="76"/>
-      <c r="O17" s="76"/>
-      <c r="P17" s="77"/>
-    </row>
-    <row r="18" spans="2:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="82" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="65" t="s">
+      <c r="D18" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="D18" s="60" t="s">
+      <c r="E18" s="65" t="s">
         <v>121</v>
       </c>
-      <c r="E18" s="60" t="s">
+      <c r="F18" s="71" t="s">
         <v>122</v>
       </c>
-      <c r="F18" s="52" t="s">
+      <c r="G18" s="90" t="s">
         <v>123</v>
       </c>
-      <c r="G18" s="73" t="s">
+      <c r="H18" s="84" t="s">
         <v>124</v>
       </c>
-      <c r="H18" s="65" t="s">
-        <v>125</v>
-      </c>
-      <c r="I18" s="68"/>
-      <c r="J18" s="60" t="s">
+      <c r="I18" s="86"/>
+      <c r="J18" s="65" t="s">
+        <v>119</v>
+      </c>
+      <c r="K18" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="K18" s="60" t="s">
+      <c r="L18" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="L18" s="52" t="s">
-        <v>122</v>
-      </c>
-      <c r="M18" s="78" t="s">
-        <v>125</v>
-      </c>
-      <c r="N18" s="60" t="s">
+      <c r="M18" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="N18" s="65" t="s">
+        <v>119</v>
+      </c>
+      <c r="O18" s="65" t="s">
         <v>120</v>
       </c>
-      <c r="O18" s="60" t="s">
+      <c r="P18" s="71" t="s">
         <v>121</v>
       </c>
-      <c r="P18" s="52" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="B19" s="83"/>
-      <c r="C19" s="66"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="74"/>
-      <c r="H19" s="69"/>
-      <c r="I19" s="64"/>
-      <c r="J19" s="61"/>
-      <c r="K19" s="61"/>
-      <c r="L19" s="53"/>
-      <c r="M19" s="66"/>
-      <c r="N19" s="61"/>
-      <c r="O19" s="61"/>
-      <c r="P19" s="53"/>
-    </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="57"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="72"/>
+      <c r="G19" s="91"/>
+      <c r="H19" s="87"/>
+      <c r="I19" s="83"/>
+      <c r="J19" s="66"/>
+      <c r="K19" s="66"/>
+      <c r="L19" s="72"/>
+      <c r="M19" s="77"/>
+      <c r="N19" s="66"/>
+      <c r="O19" s="66"/>
+      <c r="P19" s="72"/>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="42" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" s="38">
         <v>6</v>
@@ -3615,10 +3615,10 @@
       </c>
       <c r="F20" s="41"/>
       <c r="G20" s="46"/>
-      <c r="H20" s="79" t="s">
-        <v>126</v>
-      </c>
-      <c r="I20" s="55"/>
+      <c r="H20" s="52" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" s="53"/>
       <c r="J20" s="2">
         <v>3</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N20" s="2">
         <v>5</v>
@@ -3641,11 +3641,31 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="M21" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="F4:L4"/>
+    <mergeCell ref="H18:I19"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H17:L17"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:O19"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="P18:P19"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="B18:B19"/>
@@ -3662,26 +3682,6 @@
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="K12:L12"/>
     <mergeCell ref="D18:D19"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:O19"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="P18:P19"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="F4:L4"/>
-    <mergeCell ref="H18:I19"/>
-    <mergeCell ref="K13:L13"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H17:L17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>